<commit_message>
Pruebo predicciones cuando no hay partidos en  los ultimos dias
</commit_message>
<xml_diff>
--- a/p6_deployment/data/england/data_preparation/df_etiquetas_actualizado.xlsx
+++ b/p6_deployment/data/england/data_preparation/df_etiquetas_actualizado.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2786"/>
+  <dimension ref="A1:C3071"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42140,6 +42140,3468 @@
         <v>426</v>
       </c>
     </row>
+    <row r="2787">
+      <c r="A2787" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2787" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bond d 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2787" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2788">
+      <c r="A2788" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2788" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bond d 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2788" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2789">
+      <c r="A2789" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2789" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kavanagh c 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2789" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2790">
+      <c r="A2790" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2790" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pawson c 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2790" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2791">
+      <c r="A2791" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2791" t="inlineStr">
+        <is>
+          <t xml:space="preserve">brooks j 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2791" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2792">
+      <c r="A2792" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2792" t="inlineStr">
+        <is>
+          <t xml:space="preserve">taylor a 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2792" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2793">
+      <c r="A2793" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2793" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kavanagh c 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2793" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2794">
+      <c r="A2794" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2794" t="inlineStr">
+        <is>
+          <t xml:space="preserve">donohue m 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2794" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2795">
+      <c r="A2795" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2795" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bell j 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2795" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2796">
+      <c r="A2796" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2796" t="inlineStr"/>
+      <c r="C2796" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2797">
+      <c r="A2797" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2797" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ward g 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2797" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2798">
+      <c r="A2798" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2798" t="inlineStr"/>
+      <c r="C2798" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2799">
+      <c r="A2799" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2799" t="inlineStr"/>
+      <c r="C2799" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2800">
+      <c r="A2800" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2800" t="inlineStr"/>
+      <c r="C2800" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2801">
+      <c r="A2801" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2801" t="inlineStr"/>
+      <c r="C2801" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2802">
+      <c r="A2802" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2802" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ward g 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2802" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2803">
+      <c r="A2803" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2803" t="inlineStr"/>
+      <c r="C2803" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2804">
+      <c r="A2804" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2804" t="inlineStr"/>
+      <c r="C2804" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2805">
+      <c r="A2805" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2805" t="inlineStr"/>
+      <c r="C2805" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2806">
+      <c r="A2806" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2806" t="inlineStr"/>
+      <c r="C2806" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2807">
+      <c r="A2807" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2807" t="inlineStr"/>
+      <c r="C2807" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2808">
+      <c r="A2808" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2808" t="inlineStr"/>
+      <c r="C2808" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2809">
+      <c r="A2809" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2809" t="inlineStr"/>
+      <c r="C2809" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2810">
+      <c r="A2810" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2810" t="inlineStr">
+        <is>
+          <t xml:space="preserve">eltringham g 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2810" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2811">
+      <c r="A2811" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2811" t="inlineStr"/>
+      <c r="C2811" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2812">
+      <c r="A2812" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2812" t="inlineStr"/>
+      <c r="C2812" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2813">
+      <c r="A2813" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2813" t="inlineStr">
+        <is>
+          <t xml:space="preserve">smith j 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2813" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2814">
+      <c r="A2814" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2814" t="inlineStr"/>
+      <c r="C2814" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2815">
+      <c r="A2815" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2815" t="inlineStr"/>
+      <c r="C2815" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2816">
+      <c r="A2816" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2816" t="inlineStr"/>
+      <c r="C2816" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2817">
+      <c r="A2817" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2817" t="inlineStr">
+        <is>
+          <t xml:space="preserve">smith j 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2817" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2818">
+      <c r="A2818" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2818" t="inlineStr"/>
+      <c r="C2818" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2819">
+      <c r="A2819" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2819" t="inlineStr"/>
+      <c r="C2819" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2820">
+      <c r="A2820" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2820" t="inlineStr">
+        <is>
+          <t xml:space="preserve">robinson t 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2820" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2821">
+      <c r="A2821" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2821" t="inlineStr"/>
+      <c r="C2821" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2822">
+      <c r="A2822" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2822" t="inlineStr">
+        <is>
+          <t xml:space="preserve">langford o 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2822" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2823">
+      <c r="A2823" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2823" t="inlineStr"/>
+      <c r="C2823" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2824">
+      <c r="A2824" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2824" t="inlineStr"/>
+      <c r="C2824" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2825">
+      <c r="A2825" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2825" t="inlineStr"/>
+      <c r="C2825" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2826">
+      <c r="A2826" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2826" t="inlineStr"/>
+      <c r="C2826" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2827">
+      <c r="A2827" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2827" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kitchen a 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2827" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2828">
+      <c r="A2828" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2828" t="inlineStr"/>
+      <c r="C2828" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2829">
+      <c r="A2829" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2829" t="inlineStr">
+        <is>
+          <t xml:space="preserve">barrott s 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2829" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2830">
+      <c r="A2830" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2830" t="inlineStr">
+        <is>
+          <t xml:space="preserve">madley a 
+  eng </t>
+        </is>
+      </c>
+      <c r="C2830" t="n">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2831">
+      <c r="A2831" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2831" t="inlineStr">
+        <is>
+          <t xml:space="preserve">brentford community stadium
+  london </t>
+        </is>
+      </c>
+      <c r="C2831" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2832">
+      <c r="A2832" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2832" t="inlineStr">
+        <is>
+          <t xml:space="preserve">london stadium
+  london </t>
+        </is>
+      </c>
+      <c r="C2832" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2833">
+      <c r="A2833" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2833" t="inlineStr">
+        <is>
+          <t xml:space="preserve">emirates stadium
+  london </t>
+        </is>
+      </c>
+      <c r="C2833" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2834">
+      <c r="A2834" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2834" t="inlineStr">
+        <is>
+          <t xml:space="preserve">goodison park
+  liverpool </t>
+        </is>
+      </c>
+      <c r="C2834" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2835">
+      <c r="A2835" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2835" t="inlineStr">
+        <is>
+          <t xml:space="preserve">st  james  park
+  newcastle </t>
+        </is>
+      </c>
+      <c r="C2835" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2836">
+      <c r="A2836" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2836" t="inlineStr">
+        <is>
+          <t xml:space="preserve">city ground
+  nottingham </t>
+        </is>
+      </c>
+      <c r="C2836" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2837">
+      <c r="A2837" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2837" t="inlineStr">
+        <is>
+          <t xml:space="preserve">portman road
+  ipswich </t>
+        </is>
+      </c>
+      <c r="C2837" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2838">
+      <c r="A2838" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2838" t="inlineStr">
+        <is>
+          <t xml:space="preserve">old trafford
+  manchester </t>
+        </is>
+      </c>
+      <c r="C2838" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2839">
+      <c r="A2839" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2839" t="inlineStr">
+        <is>
+          <t xml:space="preserve">elland road
+  leeds </t>
+        </is>
+      </c>
+      <c r="C2839" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2840">
+      <c r="A2840" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2840" t="inlineStr">
+        <is>
+          <t xml:space="preserve">home park
+  plymouth </t>
+        </is>
+      </c>
+      <c r="C2840" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2841">
+      <c r="A2841" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2841" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mkm stadium
+  hull </t>
+        </is>
+      </c>
+      <c r="C2841" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2842">
+      <c r="A2842" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2842" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bramall lane
+  sheffield </t>
+        </is>
+      </c>
+      <c r="C2842" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2843">
+      <c r="A2843" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2843" t="inlineStr">
+        <is>
+          <t xml:space="preserve">carrow road
+  norwich </t>
+        </is>
+      </c>
+      <c r="C2843" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2844">
+      <c r="A2844" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2844" t="inlineStr">
+        <is>
+          <t xml:space="preserve">kassam stadium
+  oxford </t>
+        </is>
+      </c>
+      <c r="C2844" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2845">
+      <c r="A2845" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2845" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dw stadium
+  wigan </t>
+        </is>
+      </c>
+      <c r="C2845" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2846">
+      <c r="A2846" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2846" t="inlineStr">
+        <is>
+          <t xml:space="preserve">deepdale
+  preston </t>
+        </is>
+      </c>
+      <c r="C2846" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2847">
+      <c r="A2847" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2847" t="inlineStr">
+        <is>
+          <t xml:space="preserve">aesseal new york stadium
+  rotherham </t>
+        </is>
+      </c>
+      <c r="C2847" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2848">
+      <c r="A2848" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2848" t="inlineStr">
+        <is>
+          <t xml:space="preserve">lner stadium
+  lincoln </t>
+        </is>
+      </c>
+      <c r="C2848" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2849">
+      <c r="A2849" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2849" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the croud meadow
+  shrewsbury </t>
+        </is>
+      </c>
+      <c r="C2849" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2850">
+      <c r="A2850" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2850" t="inlineStr">
+        <is>
+          <t xml:space="preserve">swansea com stadium
+  swansea </t>
+        </is>
+      </c>
+      <c r="C2850" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2851">
+      <c r="A2851" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2851" t="inlineStr">
+        <is>
+          <t xml:space="preserve">prenton park
+  birkenhead </t>
+        </is>
+      </c>
+      <c r="C2851" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2852">
+      <c r="A2852" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2852" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bescot stadium
+  walsall </t>
+        </is>
+      </c>
+      <c r="C2852" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2853">
+      <c r="A2853" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2853" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vicarage road
+  watford </t>
+        </is>
+      </c>
+      <c r="C2853" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2854">
+      <c r="A2854" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2854" t="inlineStr">
+        <is>
+          <t xml:space="preserve">fratton park
+  portsmouth </t>
+        </is>
+      </c>
+      <c r="C2854" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2855">
+      <c r="A2855" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2855" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sixfields stadium
+  northampton </t>
+        </is>
+      </c>
+      <c r="C2855" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2856">
+      <c r="A2856" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2856" t="inlineStr">
+        <is>
+          <t xml:space="preserve">peninsula stadium
+  salford </t>
+        </is>
+      </c>
+      <c r="C2856" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2857">
+      <c r="A2857" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2857" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ashton gate stadium
+  bristol </t>
+        </is>
+      </c>
+      <c r="C2857" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2858">
+      <c r="A2858" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2858" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blundell park
+  cleethorpes </t>
+        </is>
+      </c>
+      <c r="C2858" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2859">
+      <c r="A2859" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2859" t="inlineStr">
+        <is>
+          <t xml:space="preserve">holker street
+  barrow in furness </t>
+        </is>
+      </c>
+      <c r="C2859" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2860">
+      <c r="A2860" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2860" t="inlineStr">
+        <is>
+          <t xml:space="preserve">toughsheet community stadium
+  bolton </t>
+        </is>
+      </c>
+      <c r="C2860" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2861">
+      <c r="A2861" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2861" t="inlineStr">
+        <is>
+          <t xml:space="preserve">abbey stadium
+  cambridge </t>
+        </is>
+      </c>
+      <c r="C2861" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2862">
+      <c r="A2862" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2862" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hayes lane
+  london </t>
+        </is>
+      </c>
+      <c r="C2862" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2863">
+      <c r="A2863" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2863" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pirelli stadium
+  burton upon trent </t>
+        </is>
+      </c>
+      <c r="C2863" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2864">
+      <c r="A2864" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2864" t="inlineStr">
+        <is>
+          <t xml:space="preserve">highbury stadium
+  fleetwood </t>
+        </is>
+      </c>
+      <c r="C2864" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2865">
+      <c r="A2865" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2865" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cardiff city stadium
+  cardiff </t>
+        </is>
+      </c>
+      <c r="C2865" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2866">
+      <c r="A2866" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2866" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the valley
+  london </t>
+        </is>
+      </c>
+      <c r="C2866" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2867">
+      <c r="A2867" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2867" t="inlineStr">
+        <is>
+          <t xml:space="preserve">colchester community stadium
+  colchester </t>
+        </is>
+      </c>
+      <c r="C2867" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2868">
+      <c r="A2868" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2868" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the broadfield stadium
+  crawley </t>
+        </is>
+      </c>
+      <c r="C2868" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2869">
+      <c r="A2869" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2869" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pride park
+  derby </t>
+        </is>
+      </c>
+      <c r="C2869" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2870">
+      <c r="A2870" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2870" t="inlineStr">
+        <is>
+          <t xml:space="preserve">john smith s stadium
+  huddersfield </t>
+        </is>
+      </c>
+      <c r="C2870" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2871">
+      <c r="A2871" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2871" t="inlineStr">
+        <is>
+          <t xml:space="preserve">edgeley park
+  stockport </t>
+        </is>
+      </c>
+      <c r="C2871" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2872">
+      <c r="A2872" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2872" t="inlineStr">
+        <is>
+          <t xml:space="preserve">brisbane road
+  london </t>
+        </is>
+      </c>
+      <c r="C2872" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2873">
+      <c r="A2873" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2873" t="inlineStr">
+        <is>
+          <t xml:space="preserve">brunton park
+  carlisle </t>
+        </is>
+      </c>
+      <c r="C2873" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2874">
+      <c r="A2874" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B2874" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wembley stadium
+  london </t>
+        </is>
+      </c>
+      <c r="C2874" t="n">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="2875">
+      <c r="A2875" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2875" t="inlineStr">
+        <is>
+          <t>8tPSZqtA</t>
+        </is>
+      </c>
+      <c r="C2875" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2876">
+      <c r="A2876" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2876" t="inlineStr">
+        <is>
+          <t>8tPSZqtA</t>
+        </is>
+      </c>
+      <c r="C2876" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2877">
+      <c r="A2877" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2877" t="inlineStr"/>
+      <c r="C2877" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2878">
+      <c r="A2878" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2878" t="inlineStr"/>
+      <c r="C2878" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2879">
+      <c r="A2879" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2879" t="inlineStr"/>
+      <c r="C2879" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2880">
+      <c r="A2880" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2880" t="inlineStr"/>
+      <c r="C2880" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2881">
+      <c r="A2881" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2881" t="inlineStr"/>
+      <c r="C2881" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2882">
+      <c r="A2882" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2882" t="inlineStr"/>
+      <c r="C2882" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2883">
+      <c r="A2883" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2883" t="inlineStr"/>
+      <c r="C2883" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2884">
+      <c r="A2884" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2884" t="inlineStr"/>
+      <c r="C2884" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2885">
+      <c r="A2885" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2885" t="inlineStr"/>
+      <c r="C2885" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2886">
+      <c r="A2886" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2886" t="inlineStr"/>
+      <c r="C2886" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2887">
+      <c r="A2887" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2887" t="inlineStr"/>
+      <c r="C2887" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2888">
+      <c r="A2888" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2888" t="inlineStr"/>
+      <c r="C2888" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2889">
+      <c r="A2889" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2889" t="inlineStr"/>
+      <c r="C2889" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2890">
+      <c r="A2890" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2890" t="inlineStr"/>
+      <c r="C2890" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2891">
+      <c r="A2891" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2891" t="inlineStr"/>
+      <c r="C2891" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2892">
+      <c r="A2892" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2892" t="inlineStr"/>
+      <c r="C2892" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2893">
+      <c r="A2893" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2893" t="inlineStr"/>
+      <c r="C2893" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2894">
+      <c r="A2894" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2894" t="inlineStr"/>
+      <c r="C2894" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2895">
+      <c r="A2895" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2895" t="inlineStr"/>
+      <c r="C2895" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2896">
+      <c r="A2896" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2896" t="inlineStr"/>
+      <c r="C2896" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2897">
+      <c r="A2897" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2897" t="inlineStr"/>
+      <c r="C2897" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2898">
+      <c r="A2898" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2898" t="inlineStr"/>
+      <c r="C2898" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2899">
+      <c r="A2899" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2899" t="inlineStr"/>
+      <c r="C2899" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2900">
+      <c r="A2900" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2900" t="inlineStr">
+        <is>
+          <t>n94TZqsm</t>
+        </is>
+      </c>
+      <c r="C2900" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2901">
+      <c r="A2901" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2901" t="inlineStr"/>
+      <c r="C2901" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2902">
+      <c r="A2902" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2902" t="inlineStr"/>
+      <c r="C2902" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2903">
+      <c r="A2903" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2903" t="inlineStr"/>
+      <c r="C2903" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2904">
+      <c r="A2904" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2904" t="inlineStr"/>
+      <c r="C2904" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2905">
+      <c r="A2905" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2905" t="inlineStr"/>
+      <c r="C2905" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2906">
+      <c r="A2906" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2906" t="inlineStr"/>
+      <c r="C2906" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2907">
+      <c r="A2907" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2907" t="inlineStr"/>
+      <c r="C2907" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2908">
+      <c r="A2908" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2908" t="inlineStr"/>
+      <c r="C2908" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2909">
+      <c r="A2909" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2909" t="inlineStr"/>
+      <c r="C2909" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2910">
+      <c r="A2910" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2910" t="inlineStr"/>
+      <c r="C2910" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2911">
+      <c r="A2911" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2911" t="inlineStr"/>
+      <c r="C2911" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2912">
+      <c r="A2912" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2912" t="inlineStr"/>
+      <c r="C2912" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2913">
+      <c r="A2913" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2913" t="inlineStr"/>
+      <c r="C2913" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2914">
+      <c r="A2914" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2914" t="inlineStr"/>
+      <c r="C2914" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2915">
+      <c r="A2915" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2915" t="inlineStr"/>
+      <c r="C2915" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2916">
+      <c r="A2916" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2916" t="inlineStr"/>
+      <c r="C2916" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2917">
+      <c r="A2917" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2917" t="inlineStr"/>
+      <c r="C2917" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2918">
+      <c r="A2918" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2918" t="inlineStr"/>
+      <c r="C2918" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2919">
+      <c r="A2919" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2919" t="inlineStr"/>
+      <c r="C2919" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2920">
+      <c r="A2920" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2920" t="inlineStr"/>
+      <c r="C2920" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2921">
+      <c r="A2921" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2921" t="inlineStr"/>
+      <c r="C2921" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2922">
+      <c r="A2922" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2922" t="inlineStr"/>
+      <c r="C2922" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2923">
+      <c r="A2923" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2923" t="inlineStr"/>
+      <c r="C2923" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2924">
+      <c r="A2924" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2924" t="inlineStr"/>
+      <c r="C2924" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2925">
+      <c r="A2925" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2925" t="inlineStr"/>
+      <c r="C2925" t="n">
+        <v>427</v>
+      </c>
+    </row>
+    <row r="2926">
+      <c r="A2926" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2926" t="inlineStr"/>
+      <c r="C2926" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2927">
+      <c r="A2927" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2927" t="inlineStr"/>
+      <c r="C2927" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2928">
+      <c r="A2928" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2928" t="inlineStr"/>
+      <c r="C2928" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2929">
+      <c r="A2929" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2929" t="inlineStr"/>
+      <c r="C2929" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2930">
+      <c r="A2930" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2930" t="inlineStr"/>
+      <c r="C2930" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2931">
+      <c r="A2931" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2931" t="inlineStr"/>
+      <c r="C2931" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2932">
+      <c r="A2932" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2932" t="inlineStr"/>
+      <c r="C2932" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2933">
+      <c r="A2933" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2933" t="inlineStr"/>
+      <c r="C2933" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2934">
+      <c r="A2934" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2934" t="inlineStr"/>
+      <c r="C2934" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2935">
+      <c r="A2935" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2935" t="inlineStr"/>
+      <c r="C2935" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2936">
+      <c r="A2936" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2936" t="inlineStr"/>
+      <c r="C2936" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2937">
+      <c r="A2937" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2937" t="inlineStr"/>
+      <c r="C2937" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2938">
+      <c r="A2938" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2938" t="inlineStr"/>
+      <c r="C2938" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2939">
+      <c r="A2939" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2939" t="inlineStr"/>
+      <c r="C2939" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2940">
+      <c r="A2940" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2940" t="inlineStr"/>
+      <c r="C2940" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2941">
+      <c r="A2941" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2941" t="inlineStr"/>
+      <c r="C2941" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2942">
+      <c r="A2942" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2942" t="inlineStr"/>
+      <c r="C2942" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2943">
+      <c r="A2943" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2943" t="inlineStr"/>
+      <c r="C2943" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2944">
+      <c r="A2944" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2944" t="inlineStr"/>
+      <c r="C2944" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2945">
+      <c r="A2945" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2945" t="inlineStr"/>
+      <c r="C2945" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2946">
+      <c r="A2946" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2946" t="inlineStr"/>
+      <c r="C2946" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2947">
+      <c r="A2947" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2947" t="inlineStr"/>
+      <c r="C2947" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2948">
+      <c r="A2948" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2948" t="inlineStr"/>
+      <c r="C2948" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2949">
+      <c r="A2949" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2949" t="inlineStr"/>
+      <c r="C2949" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2950">
+      <c r="A2950" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2950" t="inlineStr"/>
+      <c r="C2950" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="2951">
+      <c r="A2951" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2951" t="inlineStr"/>
+      <c r="C2951" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2952">
+      <c r="A2952" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2952" t="inlineStr"/>
+      <c r="C2952" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2953">
+      <c r="A2953" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2953" t="inlineStr"/>
+      <c r="C2953" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2954">
+      <c r="A2954" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2954" t="inlineStr"/>
+      <c r="C2954" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2955">
+      <c r="A2955" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2955" t="inlineStr"/>
+      <c r="C2955" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2956">
+      <c r="A2956" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2956" t="inlineStr"/>
+      <c r="C2956" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2957">
+      <c r="A2957" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2957" t="inlineStr"/>
+      <c r="C2957" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2958">
+      <c r="A2958" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2958" t="inlineStr"/>
+      <c r="C2958" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2959">
+      <c r="A2959" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2959" t="inlineStr"/>
+      <c r="C2959" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2960">
+      <c r="A2960" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2960" t="inlineStr"/>
+      <c r="C2960" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2961">
+      <c r="A2961" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2961" t="inlineStr"/>
+      <c r="C2961" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2962">
+      <c r="A2962" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2962" t="inlineStr"/>
+      <c r="C2962" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2963">
+      <c r="A2963" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2963" t="inlineStr"/>
+      <c r="C2963" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2964">
+      <c r="A2964" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2964" t="inlineStr"/>
+      <c r="C2964" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2965">
+      <c r="A2965" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2965" t="inlineStr"/>
+      <c r="C2965" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2966">
+      <c r="A2966" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2966" t="inlineStr"/>
+      <c r="C2966" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2967">
+      <c r="A2967" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2967" t="inlineStr"/>
+      <c r="C2967" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2968">
+      <c r="A2968" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2968" t="inlineStr"/>
+      <c r="C2968" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2969">
+      <c r="A2969" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2969" t="inlineStr"/>
+      <c r="C2969" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2970">
+      <c r="A2970" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2970" t="inlineStr"/>
+      <c r="C2970" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2971">
+      <c r="A2971" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2971" t="inlineStr"/>
+      <c r="C2971" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2972">
+      <c r="A2972" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2972" t="inlineStr"/>
+      <c r="C2972" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2973">
+      <c r="A2973" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B2973" t="inlineStr"/>
+      <c r="C2973" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="2974">
+      <c r="A2974" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2974" t="inlineStr"/>
+      <c r="C2974" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2975">
+      <c r="A2975" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2975" t="inlineStr"/>
+      <c r="C2975" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2976">
+      <c r="A2976" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2976" t="inlineStr"/>
+      <c r="C2976" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2977">
+      <c r="A2977" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2977" t="inlineStr"/>
+      <c r="C2977" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2978">
+      <c r="A2978" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2978" t="inlineStr"/>
+      <c r="C2978" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2979">
+      <c r="A2979" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2979" t="inlineStr"/>
+      <c r="C2979" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2980">
+      <c r="A2980" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2980" t="inlineStr"/>
+      <c r="C2980" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2981">
+      <c r="A2981" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2981" t="inlineStr"/>
+      <c r="C2981" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2982">
+      <c r="A2982" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2982" t="inlineStr"/>
+      <c r="C2982" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2983">
+      <c r="A2983" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2983" t="inlineStr"/>
+      <c r="C2983" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2984">
+      <c r="A2984" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2984" t="inlineStr"/>
+      <c r="C2984" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2985">
+      <c r="A2985" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2985" t="inlineStr"/>
+      <c r="C2985" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2986">
+      <c r="A2986" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2986" t="inlineStr"/>
+      <c r="C2986" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2987">
+      <c r="A2987" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2987" t="inlineStr"/>
+      <c r="C2987" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2988">
+      <c r="A2988" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2988" t="inlineStr"/>
+      <c r="C2988" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2989">
+      <c r="A2989" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2989" t="inlineStr"/>
+      <c r="C2989" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2990">
+      <c r="A2990" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2990" t="inlineStr"/>
+      <c r="C2990" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2991">
+      <c r="A2991" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2991" t="inlineStr"/>
+      <c r="C2991" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2992">
+      <c r="A2992" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2992" t="inlineStr"/>
+      <c r="C2992" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2993">
+      <c r="A2993" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2993" t="inlineStr"/>
+      <c r="C2993" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2994">
+      <c r="A2994" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2994" t="inlineStr"/>
+      <c r="C2994" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2995">
+      <c r="A2995" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2995" t="inlineStr"/>
+      <c r="C2995" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2996">
+      <c r="A2996" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2996" t="inlineStr"/>
+      <c r="C2996" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2997">
+      <c r="A2997" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2997" t="inlineStr"/>
+      <c r="C2997" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2998">
+      <c r="A2998" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B2998" t="inlineStr"/>
+      <c r="C2998" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="2999">
+      <c r="A2999" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B2999" t="inlineStr"/>
+      <c r="C2999" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3000">
+      <c r="A3000" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3000" t="inlineStr"/>
+      <c r="C3000" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3001">
+      <c r="A3001" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3001" t="inlineStr"/>
+      <c r="C3001" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3002">
+      <c r="A3002" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3002" t="inlineStr"/>
+      <c r="C3002" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3003">
+      <c r="A3003" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3003" t="inlineStr"/>
+      <c r="C3003" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3004">
+      <c r="A3004" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3004" t="inlineStr"/>
+      <c r="C3004" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3005">
+      <c r="A3005" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3005" t="inlineStr"/>
+      <c r="C3005" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3006">
+      <c r="A3006" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3006" t="inlineStr"/>
+      <c r="C3006" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3007">
+      <c r="A3007" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3007" t="inlineStr"/>
+      <c r="C3007" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3008">
+      <c r="A3008" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3008" t="inlineStr"/>
+      <c r="C3008" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3009">
+      <c r="A3009" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3009" t="inlineStr"/>
+      <c r="C3009" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3010">
+      <c r="A3010" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3010" t="inlineStr"/>
+      <c r="C3010" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3011">
+      <c r="A3011" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3011" t="inlineStr"/>
+      <c r="C3011" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3012">
+      <c r="A3012" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3012" t="inlineStr"/>
+      <c r="C3012" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3013">
+      <c r="A3013" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3013" t="inlineStr"/>
+      <c r="C3013" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3014">
+      <c r="A3014" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3014" t="inlineStr"/>
+      <c r="C3014" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3015">
+      <c r="A3015" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3015" t="inlineStr"/>
+      <c r="C3015" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3016">
+      <c r="A3016" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3016" t="inlineStr"/>
+      <c r="C3016" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3017">
+      <c r="A3017" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3017" t="inlineStr"/>
+      <c r="C3017" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3018">
+      <c r="A3018" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3018" t="inlineStr"/>
+      <c r="C3018" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3019">
+      <c r="A3019" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3019" t="inlineStr"/>
+      <c r="C3019" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3020">
+      <c r="A3020" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3020" t="inlineStr"/>
+      <c r="C3020" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3021">
+      <c r="A3021" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3021" t="inlineStr"/>
+      <c r="C3021" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3022">
+      <c r="A3022" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3022" t="inlineStr"/>
+      <c r="C3022" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3023">
+      <c r="A3023" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3023" t="inlineStr"/>
+      <c r="C3023" t="n">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="3024">
+      <c r="A3024" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3024" t="inlineStr"/>
+      <c r="C3024" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3025">
+      <c r="A3025" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3025" t="inlineStr"/>
+      <c r="C3025" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3026">
+      <c r="A3026" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3026" t="inlineStr"/>
+      <c r="C3026" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3027">
+      <c r="A3027" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3027" t="inlineStr"/>
+      <c r="C3027" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3028">
+      <c r="A3028" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3028" t="inlineStr"/>
+      <c r="C3028" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3029">
+      <c r="A3029" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3029" t="inlineStr"/>
+      <c r="C3029" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3030">
+      <c r="A3030" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3030" t="inlineStr"/>
+      <c r="C3030" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3031">
+      <c r="A3031" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3031" t="inlineStr"/>
+      <c r="C3031" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3032">
+      <c r="A3032" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3032" t="inlineStr"/>
+      <c r="C3032" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3033">
+      <c r="A3033" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3033" t="inlineStr"/>
+      <c r="C3033" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3034">
+      <c r="A3034" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3034" t="inlineStr"/>
+      <c r="C3034" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3035">
+      <c r="A3035" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3035" t="inlineStr"/>
+      <c r="C3035" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3036">
+      <c r="A3036" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3036" t="inlineStr"/>
+      <c r="C3036" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3037">
+      <c r="A3037" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3037" t="inlineStr"/>
+      <c r="C3037" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3038">
+      <c r="A3038" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3038" t="inlineStr"/>
+      <c r="C3038" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3039">
+      <c r="A3039" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3039" t="inlineStr"/>
+      <c r="C3039" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3040">
+      <c r="A3040" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3040" t="inlineStr"/>
+      <c r="C3040" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3041">
+      <c r="A3041" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3041" t="inlineStr"/>
+      <c r="C3041" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3042">
+      <c r="A3042" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3042" t="inlineStr"/>
+      <c r="C3042" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3043">
+      <c r="A3043" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3043" t="inlineStr"/>
+      <c r="C3043" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3044">
+      <c r="A3044" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3044" t="inlineStr"/>
+      <c r="C3044" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3045">
+      <c r="A3045" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3045" t="inlineStr"/>
+      <c r="C3045" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3046">
+      <c r="A3046" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3046" t="inlineStr"/>
+      <c r="C3046" t="n">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="3047">
+      <c r="A3047" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3047" t="inlineStr"/>
+      <c r="C3047" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3048">
+      <c r="A3048" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3048" t="inlineStr"/>
+      <c r="C3048" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3049">
+      <c r="A3049" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3049" t="inlineStr"/>
+      <c r="C3049" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3050">
+      <c r="A3050" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3050" t="inlineStr"/>
+      <c r="C3050" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3051">
+      <c r="A3051" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3051" t="inlineStr"/>
+      <c r="C3051" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3052">
+      <c r="A3052" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3052" t="inlineStr"/>
+      <c r="C3052" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3053">
+      <c r="A3053" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3053" t="inlineStr"/>
+      <c r="C3053" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3054">
+      <c r="A3054" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3054" t="inlineStr"/>
+      <c r="C3054" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3055">
+      <c r="A3055" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3055" t="inlineStr"/>
+      <c r="C3055" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3056">
+      <c r="A3056" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3056" t="inlineStr"/>
+      <c r="C3056" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3057">
+      <c r="A3057" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3057" t="inlineStr"/>
+      <c r="C3057" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3058">
+      <c r="A3058" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3058" t="inlineStr"/>
+      <c r="C3058" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3059">
+      <c r="A3059" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3059" t="inlineStr"/>
+      <c r="C3059" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3060">
+      <c r="A3060" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3060" t="inlineStr"/>
+      <c r="C3060" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3061">
+      <c r="A3061" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3061" t="inlineStr"/>
+      <c r="C3061" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3062">
+      <c r="A3062" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3062" t="inlineStr"/>
+      <c r="C3062" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3063">
+      <c r="A3063" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3063" t="inlineStr"/>
+      <c r="C3063" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3064">
+      <c r="A3064" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3064" t="inlineStr"/>
+      <c r="C3064" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3065">
+      <c r="A3065" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3065" t="inlineStr"/>
+      <c r="C3065" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3066">
+      <c r="A3066" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3066" t="inlineStr"/>
+      <c r="C3066" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3067">
+      <c r="A3067" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3067" t="inlineStr"/>
+      <c r="C3067" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3068">
+      <c r="A3068" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3068" t="inlineStr"/>
+      <c r="C3068" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3069">
+      <c r="A3069" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3069" t="inlineStr"/>
+      <c r="C3069" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3070">
+      <c r="A3070" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3070" t="inlineStr"/>
+      <c r="C3070" t="n">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="3071">
+      <c r="A3071" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3071" t="inlineStr"/>
+      <c r="C3071" t="n">
+        <v>429</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Prediccion para proximos partidos de todas las ligas corriendo collect_predictions.py manualmente
</commit_message>
<xml_diff>
--- a/p6_deployment/data/england/data_preparation/df_etiquetas_actualizado.xlsx
+++ b/p6_deployment/data/england/data_preparation/df_etiquetas_actualizado.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3146"/>
+  <dimension ref="A1:C3454"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -46437,6 +46437,3474 @@
         <v>430</v>
       </c>
     </row>
+    <row r="3147">
+      <c r="A3147" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3147" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hooper s 
+  eng </t>
+        </is>
+      </c>
+      <c r="C3147" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3148">
+      <c r="A3148" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3148" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hooper s 
+  eng </t>
+        </is>
+      </c>
+      <c r="C3148" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3149">
+      <c r="A3149" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3149" t="inlineStr">
+        <is>
+          <t xml:space="preserve">oliver m 
+  eng </t>
+        </is>
+      </c>
+      <c r="C3149" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3150">
+      <c r="A3150" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3150" t="inlineStr">
+        <is>
+          <t xml:space="preserve">hooper s 
+  eng </t>
+        </is>
+      </c>
+      <c r="C3150" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3151">
+      <c r="A3151" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3151" t="inlineStr">
+        <is>
+          <t xml:space="preserve">scott g 
+  eng </t>
+        </is>
+      </c>
+      <c r="C3151" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3152">
+      <c r="A3152" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3152" t="inlineStr">
+        <is>
+          <t xml:space="preserve">oliver m 
+  eng </t>
+        </is>
+      </c>
+      <c r="C3152" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3153">
+      <c r="A3153" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3153" t="inlineStr"/>
+      <c r="C3153" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3154">
+      <c r="A3154" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3154" t="inlineStr"/>
+      <c r="C3154" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3155">
+      <c r="A3155" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3155" t="inlineStr"/>
+      <c r="C3155" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3156">
+      <c r="A3156" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3156" t="inlineStr"/>
+      <c r="C3156" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3157">
+      <c r="A3157" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3157" t="inlineStr"/>
+      <c r="C3157" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3158">
+      <c r="A3158" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3158" t="inlineStr"/>
+      <c r="C3158" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3159">
+      <c r="A3159" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3159" t="inlineStr"/>
+      <c r="C3159" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3160">
+      <c r="A3160" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3160" t="inlineStr"/>
+      <c r="C3160" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3161">
+      <c r="A3161" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3161" t="inlineStr"/>
+      <c r="C3161" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3162">
+      <c r="A3162" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3162" t="inlineStr"/>
+      <c r="C3162" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3163">
+      <c r="A3163" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3163" t="inlineStr"/>
+      <c r="C3163" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3164">
+      <c r="A3164" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3164" t="inlineStr"/>
+      <c r="C3164" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3165">
+      <c r="A3165" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3165" t="inlineStr"/>
+      <c r="C3165" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3166">
+      <c r="A3166" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3166" t="inlineStr"/>
+      <c r="C3166" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3167">
+      <c r="A3167" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3167" t="inlineStr"/>
+      <c r="C3167" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3168">
+      <c r="A3168" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3168" t="inlineStr"/>
+      <c r="C3168" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3169">
+      <c r="A3169" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3169" t="inlineStr"/>
+      <c r="C3169" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3170">
+      <c r="A3170" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3170" t="inlineStr"/>
+      <c r="C3170" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3171">
+      <c r="A3171" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3171" t="inlineStr"/>
+      <c r="C3171" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3172">
+      <c r="A3172" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3172" t="inlineStr"/>
+      <c r="C3172" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3173">
+      <c r="A3173" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3173" t="inlineStr"/>
+      <c r="C3173" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3174">
+      <c r="A3174" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3174" t="inlineStr"/>
+      <c r="C3174" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3175">
+      <c r="A3175" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3175" t="inlineStr"/>
+      <c r="C3175" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3176">
+      <c r="A3176" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3176" t="inlineStr"/>
+      <c r="C3176" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3177">
+      <c r="A3177" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3177" t="inlineStr"/>
+      <c r="C3177" t="n">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="3178">
+      <c r="A3178" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B3178" t="inlineStr">
+        <is>
+          <t xml:space="preserve">anfield
+  liverpool </t>
+        </is>
+      </c>
+      <c r="C3178" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3179">
+      <c r="A3179" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B3179" t="inlineStr">
+        <is>
+          <t xml:space="preserve">vitality stadium
+  bournemouth </t>
+        </is>
+      </c>
+      <c r="C3179" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3180">
+      <c r="A3180" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B3180" t="inlineStr">
+        <is>
+          <t xml:space="preserve">molineux stadium
+  wolverhampton </t>
+        </is>
+      </c>
+      <c r="C3180" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3181">
+      <c r="A3181" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B3181" t="inlineStr">
+        <is>
+          <t xml:space="preserve">villa park
+  birmingham </t>
+        </is>
+      </c>
+      <c r="C3181" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3182">
+      <c r="A3182" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B3182" t="inlineStr">
+        <is>
+          <t xml:space="preserve">selhurst park
+  london </t>
+        </is>
+      </c>
+      <c r="C3182" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3183">
+      <c r="A3183" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B3183" t="inlineStr">
+        <is>
+          <t xml:space="preserve">craven cottage
+  london </t>
+        </is>
+      </c>
+      <c r="C3183" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3184">
+      <c r="A3184" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B3184" t="inlineStr">
+        <is>
+          <t xml:space="preserve">etihad stadium
+  manchester </t>
+        </is>
+      </c>
+      <c r="C3184" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3185">
+      <c r="A3185" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B3185" t="inlineStr">
+        <is>
+          <t xml:space="preserve">st  mary s stadium
+  southampton </t>
+        </is>
+      </c>
+      <c r="C3185" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3186">
+      <c r="A3186" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B3186" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tottenham hotspur stadium
+  london </t>
+        </is>
+      </c>
+      <c r="C3186" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3187">
+      <c r="A3187" t="inlineStr">
+        <is>
+          <t>venue</t>
+        </is>
+      </c>
+      <c r="B3187" t="inlineStr">
+        <is>
+          <t xml:space="preserve">amex stadium
+  brighton </t>
+        </is>
+      </c>
+      <c r="C3187" t="n">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="3188">
+      <c r="A3188" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3188" t="inlineStr"/>
+      <c r="C3188" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3189">
+      <c r="A3189" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3189" t="inlineStr"/>
+      <c r="C3189" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3190">
+      <c r="A3190" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3190" t="inlineStr"/>
+      <c r="C3190" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3191">
+      <c r="A3191" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3191" t="inlineStr"/>
+      <c r="C3191" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3192">
+      <c r="A3192" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3192" t="inlineStr"/>
+      <c r="C3192" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3193">
+      <c r="A3193" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3193" t="inlineStr"/>
+      <c r="C3193" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3194">
+      <c r="A3194" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3194" t="inlineStr"/>
+      <c r="C3194" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3195">
+      <c r="A3195" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3195" t="inlineStr"/>
+      <c r="C3195" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3196">
+      <c r="A3196" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3196" t="inlineStr"/>
+      <c r="C3196" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3197">
+      <c r="A3197" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3197" t="inlineStr"/>
+      <c r="C3197" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3198">
+      <c r="A3198" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3198" t="inlineStr"/>
+      <c r="C3198" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3199">
+      <c r="A3199" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3199" t="inlineStr"/>
+      <c r="C3199" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3200">
+      <c r="A3200" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3200" t="inlineStr"/>
+      <c r="C3200" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3201">
+      <c r="A3201" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3201" t="inlineStr"/>
+      <c r="C3201" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3202">
+      <c r="A3202" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3202" t="inlineStr"/>
+      <c r="C3202" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3203">
+      <c r="A3203" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3203" t="inlineStr"/>
+      <c r="C3203" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3204">
+      <c r="A3204" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3204" t="inlineStr"/>
+      <c r="C3204" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3205">
+      <c r="A3205" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3205" t="inlineStr"/>
+      <c r="C3205" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3206">
+      <c r="A3206" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3206" t="inlineStr"/>
+      <c r="C3206" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3207">
+      <c r="A3207" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3207" t="inlineStr"/>
+      <c r="C3207" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3208">
+      <c r="A3208" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3208" t="inlineStr"/>
+      <c r="C3208" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3209">
+      <c r="A3209" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3209" t="inlineStr"/>
+      <c r="C3209" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3210">
+      <c r="A3210" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3210" t="inlineStr"/>
+      <c r="C3210" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3211">
+      <c r="A3211" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3211" t="inlineStr"/>
+      <c r="C3211" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3212">
+      <c r="A3212" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3212" t="inlineStr"/>
+      <c r="C3212" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3213">
+      <c r="A3213" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3213" t="inlineStr"/>
+      <c r="C3213" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3214">
+      <c r="A3214" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3214" t="inlineStr"/>
+      <c r="C3214" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3215">
+      <c r="A3215" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3215" t="inlineStr"/>
+      <c r="C3215" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3216">
+      <c r="A3216" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3216" t="inlineStr"/>
+      <c r="C3216" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3217">
+      <c r="A3217" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3217" t="inlineStr"/>
+      <c r="C3217" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3218">
+      <c r="A3218" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3218" t="inlineStr"/>
+      <c r="C3218" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3219">
+      <c r="A3219" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3219" t="inlineStr"/>
+      <c r="C3219" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3220">
+      <c r="A3220" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3220" t="inlineStr"/>
+      <c r="C3220" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3221">
+      <c r="A3221" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3221" t="inlineStr"/>
+      <c r="C3221" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3222">
+      <c r="A3222" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3222" t="inlineStr"/>
+      <c r="C3222" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3223">
+      <c r="A3223" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3223" t="inlineStr"/>
+      <c r="C3223" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3224">
+      <c r="A3224" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3224" t="inlineStr"/>
+      <c r="C3224" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3225">
+      <c r="A3225" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3225" t="inlineStr"/>
+      <c r="C3225" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3226">
+      <c r="A3226" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3226" t="inlineStr"/>
+      <c r="C3226" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3227">
+      <c r="A3227" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3227" t="inlineStr"/>
+      <c r="C3227" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3228">
+      <c r="A3228" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3228" t="inlineStr"/>
+      <c r="C3228" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3229">
+      <c r="A3229" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3229" t="inlineStr"/>
+      <c r="C3229" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3230">
+      <c r="A3230" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3230" t="inlineStr"/>
+      <c r="C3230" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3231">
+      <c r="A3231" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3231" t="inlineStr"/>
+      <c r="C3231" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3232">
+      <c r="A3232" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3232" t="inlineStr"/>
+      <c r="C3232" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3233">
+      <c r="A3233" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3233" t="inlineStr"/>
+      <c r="C3233" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3234">
+      <c r="A3234" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3234" t="inlineStr"/>
+      <c r="C3234" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3235">
+      <c r="A3235" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3235" t="inlineStr"/>
+      <c r="C3235" t="n">
+        <v>431</v>
+      </c>
+    </row>
+    <row r="3236">
+      <c r="A3236" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3236" t="inlineStr"/>
+      <c r="C3236" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3237">
+      <c r="A3237" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3237" t="inlineStr"/>
+      <c r="C3237" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3238">
+      <c r="A3238" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3238" t="inlineStr"/>
+      <c r="C3238" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3239">
+      <c r="A3239" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3239" t="inlineStr"/>
+      <c r="C3239" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3240">
+      <c r="A3240" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3240" t="inlineStr"/>
+      <c r="C3240" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3241">
+      <c r="A3241" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3241" t="inlineStr"/>
+      <c r="C3241" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3242">
+      <c r="A3242" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3242" t="inlineStr"/>
+      <c r="C3242" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3243">
+      <c r="A3243" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3243" t="inlineStr"/>
+      <c r="C3243" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3244">
+      <c r="A3244" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3244" t="inlineStr"/>
+      <c r="C3244" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3245">
+      <c r="A3245" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3245" t="inlineStr"/>
+      <c r="C3245" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3246">
+      <c r="A3246" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3246" t="inlineStr"/>
+      <c r="C3246" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3247">
+      <c r="A3247" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3247" t="inlineStr"/>
+      <c r="C3247" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3248">
+      <c r="A3248" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3248" t="inlineStr"/>
+      <c r="C3248" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3249">
+      <c r="A3249" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3249" t="inlineStr"/>
+      <c r="C3249" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3250">
+      <c r="A3250" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3250" t="inlineStr"/>
+      <c r="C3250" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3251">
+      <c r="A3251" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3251" t="inlineStr"/>
+      <c r="C3251" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3252">
+      <c r="A3252" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3252" t="inlineStr"/>
+      <c r="C3252" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3253">
+      <c r="A3253" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3253" t="inlineStr"/>
+      <c r="C3253" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3254">
+      <c r="A3254" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3254" t="inlineStr"/>
+      <c r="C3254" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3255">
+      <c r="A3255" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3255" t="inlineStr"/>
+      <c r="C3255" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3256">
+      <c r="A3256" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3256" t="inlineStr"/>
+      <c r="C3256" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3257">
+      <c r="A3257" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3257" t="inlineStr"/>
+      <c r="C3257" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3258">
+      <c r="A3258" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3258" t="inlineStr"/>
+      <c r="C3258" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3259">
+      <c r="A3259" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3259" t="inlineStr"/>
+      <c r="C3259" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3260">
+      <c r="A3260" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3260" t="inlineStr"/>
+      <c r="C3260" t="n">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="3261">
+      <c r="A3261" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3261" t="inlineStr"/>
+      <c r="C3261" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3262">
+      <c r="A3262" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3262" t="inlineStr"/>
+      <c r="C3262" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3263">
+      <c r="A3263" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3263" t="inlineStr"/>
+      <c r="C3263" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3264">
+      <c r="A3264" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3264" t="inlineStr"/>
+      <c r="C3264" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3265">
+      <c r="A3265" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3265" t="inlineStr"/>
+      <c r="C3265" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3266">
+      <c r="A3266" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3266" t="inlineStr"/>
+      <c r="C3266" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3267">
+      <c r="A3267" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3267" t="inlineStr"/>
+      <c r="C3267" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3268">
+      <c r="A3268" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3268" t="inlineStr"/>
+      <c r="C3268" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3269">
+      <c r="A3269" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3269" t="inlineStr"/>
+      <c r="C3269" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3270">
+      <c r="A3270" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3270" t="inlineStr"/>
+      <c r="C3270" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3271">
+      <c r="A3271" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3271" t="inlineStr"/>
+      <c r="C3271" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3272">
+      <c r="A3272" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3272" t="inlineStr"/>
+      <c r="C3272" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3273">
+      <c r="A3273" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3273" t="inlineStr"/>
+      <c r="C3273" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3274">
+      <c r="A3274" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3274" t="inlineStr"/>
+      <c r="C3274" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3275">
+      <c r="A3275" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3275" t="inlineStr"/>
+      <c r="C3275" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3276">
+      <c r="A3276" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3276" t="inlineStr"/>
+      <c r="C3276" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3277">
+      <c r="A3277" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3277" t="inlineStr"/>
+      <c r="C3277" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3278">
+      <c r="A3278" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3278" t="inlineStr"/>
+      <c r="C3278" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3279">
+      <c r="A3279" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3279" t="inlineStr"/>
+      <c r="C3279" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3280">
+      <c r="A3280" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3280" t="inlineStr"/>
+      <c r="C3280" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3281">
+      <c r="A3281" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3281" t="inlineStr"/>
+      <c r="C3281" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3282">
+      <c r="A3282" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3282" t="inlineStr"/>
+      <c r="C3282" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3283">
+      <c r="A3283" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3283" t="inlineStr"/>
+      <c r="C3283" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3284">
+      <c r="A3284" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3284" t="inlineStr"/>
+      <c r="C3284" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3285">
+      <c r="A3285" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3285" t="inlineStr"/>
+      <c r="C3285" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3286">
+      <c r="A3286" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3286" t="inlineStr"/>
+      <c r="C3286" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3287">
+      <c r="A3287" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3287" t="inlineStr"/>
+      <c r="C3287" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3288">
+      <c r="A3288" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3288" t="inlineStr"/>
+      <c r="C3288" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3289">
+      <c r="A3289" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3289" t="inlineStr"/>
+      <c r="C3289" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3290">
+      <c r="A3290" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3290" t="inlineStr"/>
+      <c r="C3290" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3291">
+      <c r="A3291" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3291" t="inlineStr"/>
+      <c r="C3291" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3292">
+      <c r="A3292" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3292" t="inlineStr"/>
+      <c r="C3292" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3293">
+      <c r="A3293" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3293" t="inlineStr"/>
+      <c r="C3293" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3294">
+      <c r="A3294" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3294" t="inlineStr"/>
+      <c r="C3294" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3295">
+      <c r="A3295" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3295" t="inlineStr"/>
+      <c r="C3295" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3296">
+      <c r="A3296" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3296" t="inlineStr"/>
+      <c r="C3296" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3297">
+      <c r="A3297" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3297" t="inlineStr"/>
+      <c r="C3297" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3298">
+      <c r="A3298" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3298" t="inlineStr"/>
+      <c r="C3298" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3299">
+      <c r="A3299" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3299" t="inlineStr"/>
+      <c r="C3299" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3300">
+      <c r="A3300" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3300" t="inlineStr"/>
+      <c r="C3300" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3301">
+      <c r="A3301" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3301" t="inlineStr"/>
+      <c r="C3301" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3302">
+      <c r="A3302" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3302" t="inlineStr"/>
+      <c r="C3302" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3303">
+      <c r="A3303" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3303" t="inlineStr"/>
+      <c r="C3303" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3304">
+      <c r="A3304" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3304" t="inlineStr"/>
+      <c r="C3304" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3305">
+      <c r="A3305" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3305" t="inlineStr"/>
+      <c r="C3305" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3306">
+      <c r="A3306" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3306" t="inlineStr"/>
+      <c r="C3306" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3307">
+      <c r="A3307" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3307" t="inlineStr"/>
+      <c r="C3307" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3308">
+      <c r="A3308" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3308" t="inlineStr"/>
+      <c r="C3308" t="n">
+        <v>432</v>
+      </c>
+    </row>
+    <row r="3309">
+      <c r="A3309" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3309" t="inlineStr"/>
+      <c r="C3309" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3310">
+      <c r="A3310" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3310" t="inlineStr"/>
+      <c r="C3310" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3311">
+      <c r="A3311" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3311" t="inlineStr"/>
+      <c r="C3311" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3312">
+      <c r="A3312" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3312" t="inlineStr"/>
+      <c r="C3312" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3313">
+      <c r="A3313" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3313" t="inlineStr"/>
+      <c r="C3313" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3314">
+      <c r="A3314" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3314" t="inlineStr"/>
+      <c r="C3314" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3315">
+      <c r="A3315" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3315" t="inlineStr"/>
+      <c r="C3315" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3316">
+      <c r="A3316" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3316" t="inlineStr"/>
+      <c r="C3316" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3317">
+      <c r="A3317" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3317" t="inlineStr"/>
+      <c r="C3317" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3318">
+      <c r="A3318" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3318" t="inlineStr"/>
+      <c r="C3318" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3319">
+      <c r="A3319" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3319" t="inlineStr"/>
+      <c r="C3319" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3320">
+      <c r="A3320" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3320" t="inlineStr"/>
+      <c r="C3320" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3321">
+      <c r="A3321" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3321" t="inlineStr"/>
+      <c r="C3321" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3322">
+      <c r="A3322" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3322" t="inlineStr"/>
+      <c r="C3322" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3323">
+      <c r="A3323" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3323" t="inlineStr"/>
+      <c r="C3323" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3324">
+      <c r="A3324" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3324" t="inlineStr"/>
+      <c r="C3324" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3325">
+      <c r="A3325" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3325" t="inlineStr"/>
+      <c r="C3325" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3326">
+      <c r="A3326" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3326" t="inlineStr"/>
+      <c r="C3326" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3327">
+      <c r="A3327" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3327" t="inlineStr"/>
+      <c r="C3327" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3328">
+      <c r="A3328" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3328" t="inlineStr"/>
+      <c r="C3328" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3329">
+      <c r="A3329" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3329" t="inlineStr"/>
+      <c r="C3329" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3330">
+      <c r="A3330" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3330" t="inlineStr"/>
+      <c r="C3330" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3331">
+      <c r="A3331" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3331" t="inlineStr"/>
+      <c r="C3331" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3332">
+      <c r="A3332" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3332" t="inlineStr"/>
+      <c r="C3332" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3333">
+      <c r="A3333" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3333" t="inlineStr"/>
+      <c r="C3333" t="n">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="3334">
+      <c r="A3334" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3334" t="inlineStr"/>
+      <c r="C3334" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3335">
+      <c r="A3335" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3335" t="inlineStr"/>
+      <c r="C3335" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3336">
+      <c r="A3336" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3336" t="inlineStr"/>
+      <c r="C3336" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3337">
+      <c r="A3337" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3337" t="inlineStr"/>
+      <c r="C3337" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3338">
+      <c r="A3338" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3338" t="inlineStr"/>
+      <c r="C3338" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3339">
+      <c r="A3339" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3339" t="inlineStr"/>
+      <c r="C3339" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3340">
+      <c r="A3340" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3340" t="inlineStr"/>
+      <c r="C3340" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3341">
+      <c r="A3341" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3341" t="inlineStr"/>
+      <c r="C3341" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3342">
+      <c r="A3342" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3342" t="inlineStr"/>
+      <c r="C3342" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3343">
+      <c r="A3343" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3343" t="inlineStr"/>
+      <c r="C3343" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3344">
+      <c r="A3344" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3344" t="inlineStr"/>
+      <c r="C3344" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3345">
+      <c r="A3345" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3345" t="inlineStr"/>
+      <c r="C3345" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3346">
+      <c r="A3346" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3346" t="inlineStr"/>
+      <c r="C3346" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3347">
+      <c r="A3347" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3347" t="inlineStr"/>
+      <c r="C3347" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3348">
+      <c r="A3348" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3348" t="inlineStr"/>
+      <c r="C3348" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3349">
+      <c r="A3349" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3349" t="inlineStr"/>
+      <c r="C3349" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3350">
+      <c r="A3350" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3350" t="inlineStr"/>
+      <c r="C3350" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3351">
+      <c r="A3351" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3351" t="inlineStr"/>
+      <c r="C3351" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3352">
+      <c r="A3352" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3352" t="inlineStr"/>
+      <c r="C3352" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3353">
+      <c r="A3353" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3353" t="inlineStr"/>
+      <c r="C3353" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3354">
+      <c r="A3354" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3354" t="inlineStr"/>
+      <c r="C3354" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3355">
+      <c r="A3355" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3355" t="inlineStr"/>
+      <c r="C3355" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3356">
+      <c r="A3356" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3356" t="inlineStr"/>
+      <c r="C3356" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3357">
+      <c r="A3357" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3357" t="inlineStr"/>
+      <c r="C3357" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3358">
+      <c r="A3358" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3358" t="inlineStr"/>
+      <c r="C3358" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3359">
+      <c r="A3359" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3359" t="inlineStr"/>
+      <c r="C3359" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3360">
+      <c r="A3360" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3360" t="inlineStr"/>
+      <c r="C3360" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3361">
+      <c r="A3361" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3361" t="inlineStr"/>
+      <c r="C3361" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3362">
+      <c r="A3362" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3362" t="inlineStr"/>
+      <c r="C3362" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3363">
+      <c r="A3363" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3363" t="inlineStr"/>
+      <c r="C3363" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3364">
+      <c r="A3364" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3364" t="inlineStr"/>
+      <c r="C3364" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3365">
+      <c r="A3365" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3365" t="inlineStr"/>
+      <c r="C3365" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3366">
+      <c r="A3366" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3366" t="inlineStr"/>
+      <c r="C3366" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3367">
+      <c r="A3367" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3367" t="inlineStr"/>
+      <c r="C3367" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3368">
+      <c r="A3368" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3368" t="inlineStr"/>
+      <c r="C3368" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3369">
+      <c r="A3369" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3369" t="inlineStr"/>
+      <c r="C3369" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3370">
+      <c r="A3370" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3370" t="inlineStr"/>
+      <c r="C3370" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3371">
+      <c r="A3371" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3371" t="inlineStr"/>
+      <c r="C3371" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3372">
+      <c r="A3372" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3372" t="inlineStr"/>
+      <c r="C3372" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3373">
+      <c r="A3373" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3373" t="inlineStr"/>
+      <c r="C3373" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3374">
+      <c r="A3374" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3374" t="inlineStr"/>
+      <c r="C3374" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3375">
+      <c r="A3375" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3375" t="inlineStr"/>
+      <c r="C3375" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3376">
+      <c r="A3376" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3376" t="inlineStr"/>
+      <c r="C3376" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3377">
+      <c r="A3377" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3377" t="inlineStr"/>
+      <c r="C3377" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3378">
+      <c r="A3378" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3378" t="inlineStr"/>
+      <c r="C3378" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3379">
+      <c r="A3379" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3379" t="inlineStr"/>
+      <c r="C3379" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3380">
+      <c r="A3380" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3380" t="inlineStr"/>
+      <c r="C3380" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3381">
+      <c r="A3381" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3381" t="inlineStr"/>
+      <c r="C3381" t="n">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="3382">
+      <c r="A3382" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3382" t="inlineStr"/>
+      <c r="C3382" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3383">
+      <c r="A3383" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3383" t="inlineStr"/>
+      <c r="C3383" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3384">
+      <c r="A3384" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3384" t="inlineStr"/>
+      <c r="C3384" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3385">
+      <c r="A3385" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3385" t="inlineStr"/>
+      <c r="C3385" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3386">
+      <c r="A3386" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3386" t="inlineStr"/>
+      <c r="C3386" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3387">
+      <c r="A3387" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3387" t="inlineStr"/>
+      <c r="C3387" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3388">
+      <c r="A3388" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3388" t="inlineStr"/>
+      <c r="C3388" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3389">
+      <c r="A3389" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3389" t="inlineStr"/>
+      <c r="C3389" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3390">
+      <c r="A3390" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3390" t="inlineStr"/>
+      <c r="C3390" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3391">
+      <c r="A3391" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3391" t="inlineStr"/>
+      <c r="C3391" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3392">
+      <c r="A3392" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3392" t="inlineStr"/>
+      <c r="C3392" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3393">
+      <c r="A3393" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3393" t="inlineStr"/>
+      <c r="C3393" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3394">
+      <c r="A3394" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3394" t="inlineStr"/>
+      <c r="C3394" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3395">
+      <c r="A3395" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3395" t="inlineStr"/>
+      <c r="C3395" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3396">
+      <c r="A3396" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3396" t="inlineStr"/>
+      <c r="C3396" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3397">
+      <c r="A3397" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3397" t="inlineStr"/>
+      <c r="C3397" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3398">
+      <c r="A3398" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3398" t="inlineStr"/>
+      <c r="C3398" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3399">
+      <c r="A3399" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3399" t="inlineStr"/>
+      <c r="C3399" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3400">
+      <c r="A3400" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3400" t="inlineStr"/>
+      <c r="C3400" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3401">
+      <c r="A3401" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3401" t="inlineStr"/>
+      <c r="C3401" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3402">
+      <c r="A3402" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3402" t="inlineStr"/>
+      <c r="C3402" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3403">
+      <c r="A3403" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3403" t="inlineStr"/>
+      <c r="C3403" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3404">
+      <c r="A3404" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3404" t="inlineStr"/>
+      <c r="C3404" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3405">
+      <c r="A3405" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3405" t="inlineStr"/>
+      <c r="C3405" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3406">
+      <c r="A3406" t="inlineStr">
+        <is>
+          <t>referee</t>
+        </is>
+      </c>
+      <c r="B3406" t="inlineStr"/>
+      <c r="C3406" t="n">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="3407">
+      <c r="A3407" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3407" t="inlineStr"/>
+      <c r="C3407" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3408">
+      <c r="A3408" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3408" t="inlineStr"/>
+      <c r="C3408" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3409">
+      <c r="A3409" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3409" t="inlineStr"/>
+      <c r="C3409" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3410">
+      <c r="A3410" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3410" t="inlineStr"/>
+      <c r="C3410" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3411">
+      <c r="A3411" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3411" t="inlineStr"/>
+      <c r="C3411" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3412">
+      <c r="A3412" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3412" t="inlineStr"/>
+      <c r="C3412" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3413">
+      <c r="A3413" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3413" t="inlineStr"/>
+      <c r="C3413" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3414">
+      <c r="A3414" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3414" t="inlineStr"/>
+      <c r="C3414" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3415">
+      <c r="A3415" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3415" t="inlineStr"/>
+      <c r="C3415" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3416">
+      <c r="A3416" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3416" t="inlineStr"/>
+      <c r="C3416" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3417">
+      <c r="A3417" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3417" t="inlineStr"/>
+      <c r="C3417" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3418">
+      <c r="A3418" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3418" t="inlineStr"/>
+      <c r="C3418" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3419">
+      <c r="A3419" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3419" t="inlineStr"/>
+      <c r="C3419" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3420">
+      <c r="A3420" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3420" t="inlineStr"/>
+      <c r="C3420" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3421">
+      <c r="A3421" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3421" t="inlineStr"/>
+      <c r="C3421" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3422">
+      <c r="A3422" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3422" t="inlineStr"/>
+      <c r="C3422" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3423">
+      <c r="A3423" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3423" t="inlineStr"/>
+      <c r="C3423" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3424">
+      <c r="A3424" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3424" t="inlineStr"/>
+      <c r="C3424" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3425">
+      <c r="A3425" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3425" t="inlineStr"/>
+      <c r="C3425" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3426">
+      <c r="A3426" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3426" t="inlineStr"/>
+      <c r="C3426" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3427">
+      <c r="A3427" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3427" t="inlineStr"/>
+      <c r="C3427" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3428">
+      <c r="A3428" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3428" t="inlineStr"/>
+      <c r="C3428" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3429">
+      <c r="A3429" t="inlineStr">
+        <is>
+          <t>id_coach_home</t>
+        </is>
+      </c>
+      <c r="B3429" t="inlineStr"/>
+      <c r="C3429" t="n">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="3430">
+      <c r="A3430" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3430" t="inlineStr"/>
+      <c r="C3430" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3431">
+      <c r="A3431" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3431" t="inlineStr"/>
+      <c r="C3431" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3432">
+      <c r="A3432" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3432" t="inlineStr"/>
+      <c r="C3432" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3433">
+      <c r="A3433" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3433" t="inlineStr"/>
+      <c r="C3433" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3434">
+      <c r="A3434" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3434" t="inlineStr"/>
+      <c r="C3434" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3435">
+      <c r="A3435" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3435" t="inlineStr"/>
+      <c r="C3435" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3436">
+      <c r="A3436" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3436" t="inlineStr"/>
+      <c r="C3436" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3437">
+      <c r="A3437" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3437" t="inlineStr"/>
+      <c r="C3437" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3438">
+      <c r="A3438" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3438" t="inlineStr"/>
+      <c r="C3438" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3439">
+      <c r="A3439" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3439" t="inlineStr"/>
+      <c r="C3439" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3440">
+      <c r="A3440" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3440" t="inlineStr"/>
+      <c r="C3440" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3441">
+      <c r="A3441" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3441" t="inlineStr"/>
+      <c r="C3441" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3442">
+      <c r="A3442" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3442" t="inlineStr"/>
+      <c r="C3442" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3443">
+      <c r="A3443" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3443" t="inlineStr"/>
+      <c r="C3443" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3444">
+      <c r="A3444" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3444" t="inlineStr"/>
+      <c r="C3444" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3445">
+      <c r="A3445" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3445" t="inlineStr"/>
+      <c r="C3445" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3446">
+      <c r="A3446" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3446" t="inlineStr"/>
+      <c r="C3446" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3447">
+      <c r="A3447" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3447" t="inlineStr"/>
+      <c r="C3447" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3448">
+      <c r="A3448" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3448" t="inlineStr"/>
+      <c r="C3448" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3449">
+      <c r="A3449" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3449" t="inlineStr"/>
+      <c r="C3449" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3450">
+      <c r="A3450" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3450" t="inlineStr"/>
+      <c r="C3450" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3451">
+      <c r="A3451" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3451" t="inlineStr"/>
+      <c r="C3451" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3452">
+      <c r="A3452" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3452" t="inlineStr"/>
+      <c r="C3452" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3453">
+      <c r="A3453" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3453" t="inlineStr"/>
+      <c r="C3453" t="n">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="3454">
+      <c r="A3454" t="inlineStr">
+        <is>
+          <t>id_coach_away</t>
+        </is>
+      </c>
+      <c r="B3454" t="inlineStr"/>
+      <c r="C3454" t="n">
+        <v>434</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>